<commit_message>
add Creo quote integration
</commit_message>
<xml_diff>
--- a/resources/Templates/对象系数.xlsx
+++ b/resources/Templates/对象系数.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\liuruiwen\IPXprice\IPXtest\backup\IPXQuote-mytest\IPXQuotetest\resources\Templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12375"/>
+    <workbookView windowWidth="15735" windowHeight="11250"/>
   </bookViews>
   <sheets>
     <sheet name="对象系数" sheetId="1" r:id="rId1"/>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
   <si>
     <t>类别</t>
   </si>
@@ -38,6 +43,12 @@
     <t>图纸对象系数(表中为默认值，可配置，要求数值非负)</t>
   </si>
   <si>
+    <t>SW软件系数</t>
+  </si>
+  <si>
+    <t>Creo软件系数</t>
+  </si>
+  <si>
     <t>备注</t>
   </si>
   <si>
@@ -47,13 +58,19 @@
     <t>特征</t>
   </si>
   <si>
+    <t>考虑到Creo实体化特征的复杂度，做适当系数放大</t>
+  </si>
+  <si>
+    <t>配置项</t>
+  </si>
+  <si>
+    <t>Creo对应的族表项、简化表示项、表示项</t>
+  </si>
+  <si>
+    <t>表达式</t>
+  </si>
+  <si>
     <t/>
-  </si>
-  <si>
-    <t>配置项</t>
-  </si>
-  <si>
-    <t>表达式</t>
   </si>
   <si>
     <t>装配</t>
@@ -126,11 +143,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="0.00_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -744,10 +762,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1281,16 +1300,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="16.5" outlineLevelCol="3"/>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="8" defaultRowHeight="16.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="4" max="5" width="12.1111111111111" customWidth="1"/>
+    <col min="6" max="6" width="72" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1303,245 +1323,319 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="2">
         <v>0.5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2">
         <v>0.1</v>
       </c>
-      <c r="D4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="D4" s="3">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2">
         <v>0.6</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="D5" s="3">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2">
         <v>0.8</v>
       </c>
-      <c r="D6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>9</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2">
-        <v>1</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
       </c>
       <c r="C8" s="2">
         <v>0.5</v>
       </c>
-      <c r="D8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2">
         <v>0.1</v>
       </c>
-      <c r="D9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C10" s="2">
         <v>0.8</v>
       </c>
-      <c r="D10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2">
         <v>0.5</v>
       </c>
-      <c r="D11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C12" s="2">
         <v>0.5</v>
       </c>
-      <c r="D12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B15" s="2">
-        <v>1.12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
+        <v>27</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B19" s="2">
         <v>15</v>
       </c>
       <c r="C19" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B20" s="2">
         <v>40</v>
       </c>
       <c r="C20" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D20" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2">
         <v>80</v>
       </c>
       <c r="C21" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C22" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="D22" t="s">
-        <v>6</v>
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>